<commit_message>
Disparo WhatsApp ConstruMais: empresas fora, 9 incluído, histórico atualizado
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017neZwiKZPMdbwfnz9Yzqxo
</commit_message>
<xml_diff>
--- a/Operacional/clientes/construmais/outputs/10-2026/Arquivos/14-disparo-whatsapp/14-disparo-whatsapp-lote-02.xlsx
+++ b/Operacional/clientes/construmais/outputs/10-2026/Arquivos/14-disparo-whatsapp/14-disparo-whatsapp-lote-02.xlsx
@@ -504,721 +504,721 @@
     </row>
     <row r="4">
       <c r="A4" s="4" t="n">
-        <v>5583987464446</v>
+        <v>5583997163263</v>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Manoel</t>
+          <t>Semear</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Manoel Edson Soares</t>
+          <t>Semear Sustentabilidade</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="4" t="n">
-        <v>5583988391747</v>
+        <v>5583987464446</v>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Gerlane</t>
+          <t>Manoel</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Gerlane da Silva Costa</t>
+          <t>Manoel Edson Soares</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
-        <v>5583986302777</v>
+        <v>5583988391747</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Carla</t>
+          <t>Gerlane</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Carla Maria da Silva</t>
+          <t>Gerlane da Silva Costa</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n">
-        <v>5583988542687</v>
+        <v>5583986302777</v>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Marcio</t>
+          <t>Carla</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Marcio Andre Baracho da Silva</t>
+          <t>Carla Maria da Silva</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
-        <v>5583996414931</v>
+        <v>5583988542687</v>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Matheus</t>
+          <t>Marcio</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Matheus da Silva Romao</t>
+          <t>Marcio Andre Baracho da Silva</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n">
-        <v>5583991091872</v>
+        <v>5583996414931</v>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Severino</t>
+          <t>Matheus</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Severino Ramos Marcolino Cavalcante</t>
+          <t>Matheus da Silva Romao</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="n">
-        <v>5583988872565</v>
+        <v>5583991091872</v>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Cristina</t>
+          <t>Severino</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Cristina Feitosa de Santana</t>
+          <t>Severino Ramos Marcolino Cavalcante</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n">
-        <v>5583988208756</v>
+        <v>5583988872565</v>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Lenilda</t>
+          <t>Cristina</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Lenilda Galdino Silva dos Santos</t>
+          <t>Cristina Feitosa de Santana</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="n">
-        <v>5583988100008</v>
+        <v>5583988208756</v>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Luis</t>
+          <t>Lenilda</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Luis Fernando Guedes Camargo</t>
+          <t>Lenilda Galdino Silva dos Santos</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n">
-        <v>5583996049402</v>
+        <v>5583988100008</v>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Amos</t>
+          <t>Luis</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Amos Souza Soares</t>
+          <t>Luis Fernando Guedes Camargo</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="n">
-        <v>5583988738754</v>
+        <v>5583996049402</v>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Jose</t>
+          <t>Amos</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Jose Hildo Herculano de Oliveira</t>
+          <t>Amos Souza Soares</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n">
-        <v>5583988050818</v>
+        <v>5583988738754</v>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Heverson</t>
+          <t>Jose</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Heverson Ferreira Soares</t>
+          <t>Jose Hildo Herculano de Oliveira</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="n">
-        <v>5582993311821</v>
+        <v>5583988050818</v>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Wx</t>
+          <t>Heverson</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Wx Esquadrias</t>
+          <t>Heverson Ferreira Soares</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n">
-        <v>5583988681747</v>
+        <v>5582993311821</v>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Atacarejo</t>
+          <t>Wx</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Atacarejo Atlantico Sul</t>
+          <t>Wx Esquadrias</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="n">
-        <v>5583999435773</v>
+        <v>5583988681747</v>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Francisca</t>
+          <t>Atacarejo</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Francisca Carneiro de Freitas</t>
+          <t>Atacarejo Atlantico Sul</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n">
-        <v>5583996841483</v>
+        <v>5583999435773</v>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Lucas</t>
+          <t>Francisca</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Lucas Fernandes</t>
+          <t>Francisca Carneiro de Freitas</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="n">
-        <v>5583991427155</v>
+        <v>5583996841483</v>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Lauricelia</t>
+          <t>Lucas</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Lauricelia da Silva Santana</t>
+          <t>Lucas Fernandes</t>
         </is>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" s="3">
       <c r="A21" s="4" t="n">
-        <v>5583999500110</v>
+        <v>5583991427155</v>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Jose</t>
+          <t>Lauricelia</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Jose Mauricio Barbosa Lira</t>
+          <t>Lauricelia da Silva Santana</t>
         </is>
       </c>
     </row>
     <row r="22" ht="15.75" customHeight="1" s="3">
       <c r="A22" s="4" t="n">
-        <v>5583988502373</v>
+        <v>5581971093406</v>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Carlos</t>
+          <t>Concrearte</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Carlos Alexandre Silva Diniz</t>
+          <t>Concrearte</t>
         </is>
       </c>
     </row>
     <row r="23" ht="15.75" customHeight="1" s="3">
       <c r="A23" s="4" t="n">
-        <v>5583988678355</v>
+        <v>5583999500110</v>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Laerte</t>
+          <t>Jose</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Laerte Araujo da Cruz</t>
+          <t>Jose Mauricio Barbosa Lira</t>
         </is>
       </c>
     </row>
     <row r="24" ht="15.75" customHeight="1" s="3">
       <c r="A24" s="4" t="n">
-        <v>5583998782701</v>
+        <v>5583988502373</v>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Tiago</t>
+          <t>Carlos</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Tiago Anastacio da Silva</t>
+          <t>Carlos Alexandre Silva Diniz</t>
         </is>
       </c>
     </row>
     <row r="25" ht="15.75" customHeight="1" s="3">
       <c r="A25" s="4" t="n">
-        <v>5583999824954</v>
+        <v>5583988678355</v>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Jose</t>
+          <t>Laerte</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Jose Salvino Filho</t>
+          <t>Laerte Araujo da Cruz</t>
         </is>
       </c>
     </row>
     <row r="26" ht="15.75" customHeight="1" s="3">
       <c r="A26" s="4" t="n">
-        <v>5583988599011</v>
+        <v>5583998782701</v>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Marcio</t>
+          <t>Tiago</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Marcio Muniz Andrade</t>
+          <t>Tiago Anastacio da Silva</t>
         </is>
       </c>
     </row>
     <row r="27" ht="15.75" customHeight="1" s="3">
       <c r="A27" s="4" t="n">
-        <v>5583991850422</v>
+        <v>5583999824954</v>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Conarte</t>
+          <t>Jose</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Conarte</t>
+          <t>Jose Salvino Filho</t>
         </is>
       </c>
     </row>
     <row r="28" ht="15.75" customHeight="1" s="3">
       <c r="A28" s="4" t="n">
-        <v>5583998040131</v>
+        <v>5583988599011</v>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Ruam</t>
+          <t>Marcio</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Ruam Matheus Moura de Lima</t>
+          <t>Marcio Muniz Andrade</t>
         </is>
       </c>
     </row>
     <row r="29" ht="15.75" customHeight="1" s="3">
       <c r="A29" s="4" t="n">
-        <v>5581997272299</v>
+        <v>5583991850422</v>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Leopoldo</t>
+          <t>Conarte</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Leopoldo Soares da Silva</t>
+          <t>Conarte</t>
         </is>
       </c>
     </row>
     <row r="30" ht="15.75" customHeight="1" s="3">
       <c r="A30" s="4" t="n">
-        <v>5583987702553</v>
+        <v>5583998040131</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Jose</t>
+          <t>Ruam</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Jose Mendes Brito</t>
+          <t>Ruam Matheus Moura de Lima</t>
         </is>
       </c>
     </row>
     <row r="31" ht="15.75" customHeight="1" s="3">
       <c r="A31" s="4" t="n">
-        <v>5583998187756</v>
+        <v>5581997272299</v>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Sivenildo</t>
+          <t>Leopoldo</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Sivenildo de Azevedo Batista</t>
+          <t>Leopoldo Soares da Silva</t>
         </is>
       </c>
     </row>
     <row r="32" ht="15.75" customHeight="1" s="3">
       <c r="A32" s="4" t="n">
-        <v>5583988469983</v>
+        <v>5583987702553</v>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Alexandre</t>
+          <t>Jose</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Alexandre Rodrigues da Silva</t>
+          <t>Jose Mendes Brito</t>
         </is>
       </c>
     </row>
     <row r="33" ht="15.75" customHeight="1" s="3">
       <c r="A33" s="4" t="n">
-        <v>5583981599421</v>
+        <v>5583998187756</v>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Maria</t>
+          <t>Sivenildo</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Maria Celia Henriques Alves</t>
+          <t>Sivenildo de Azevedo Batista</t>
         </is>
       </c>
     </row>
     <row r="34" ht="15.75" customHeight="1" s="3">
       <c r="A34" s="4" t="n">
-        <v>5583991490727</v>
+        <v>5583988469983</v>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Alexson</t>
+          <t>Alexandre</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Alexson Correia da Silva</t>
+          <t>Alexandre Rodrigues da Silva</t>
         </is>
       </c>
     </row>
     <row r="35" ht="15.75" customHeight="1" s="3">
       <c r="A35" s="4" t="n">
-        <v>5583991039487</v>
+        <v>5583981599421</v>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Jobilson</t>
+          <t>Maria</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Jobilson de Sousa</t>
+          <t>Maria Celia Henriques Alves</t>
         </is>
       </c>
     </row>
     <row r="36" ht="15.75" customHeight="1" s="3">
       <c r="A36" s="4" t="n">
-        <v>5583987542726</v>
+        <v>5583991490727</v>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Jose</t>
+          <t>Alexson</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Jose Douglas Cipriano</t>
+          <t>Alexson Correia da Silva</t>
         </is>
       </c>
     </row>
     <row r="37" ht="15.75" customHeight="1" s="3">
       <c r="A37" s="4" t="n">
-        <v>5583994099032</v>
+        <v>5583991039487</v>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Raquel</t>
+          <t>Jobilson</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Raquel Pires Araujo Soares</t>
+          <t>Jobilson de Sousa</t>
         </is>
       </c>
     </row>
     <row r="38" ht="15.75" customHeight="1" s="3">
       <c r="A38" s="4" t="n">
-        <v>5583987487581</v>
+        <v>5583987542726</v>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Joelson</t>
+          <t>Jose</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Joelson Oliveira da Silva</t>
+          <t>Jose Douglas Cipriano</t>
         </is>
       </c>
     </row>
     <row r="39" ht="15.75" customHeight="1" s="3">
       <c r="A39" s="4" t="n">
-        <v>5583986751910</v>
+        <v>5583994099032</v>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Gilvania</t>
+          <t>Raquel</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Gilvania Rodrigues da Silva</t>
+          <t>Raquel Pires Araujo Soares</t>
         </is>
       </c>
     </row>
     <row r="40" ht="15.75" customHeight="1" s="3">
       <c r="A40" s="4" t="n">
-        <v>5583998213093</v>
+        <v>5583987487581</v>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Wellington</t>
+          <t>Joelson</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Wellington Nascimento da Silva</t>
+          <t>Joelson Oliveira da Silva</t>
         </is>
       </c>
     </row>
     <row r="41" ht="15.75" customHeight="1" s="3">
       <c r="A41" s="4" t="n">
-        <v>5583981508768</v>
+        <v>5583986751910</v>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Samir</t>
+          <t>Gilvania</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Samir Said Castor Goncalves</t>
+          <t>Gilvania Rodrigues da Silva</t>
         </is>
       </c>
     </row>
     <row r="42" ht="15.75" customHeight="1" s="3">
       <c r="A42" s="4" t="n">
-        <v>5583993707561</v>
+        <v>5583998213093</v>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Antonio</t>
+          <t>Wellington</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Antonio Pessoa Cirino</t>
+          <t>Wellington Nascimento da Silva</t>
         </is>
       </c>
     </row>
     <row r="43" ht="15.75" customHeight="1" s="3">
       <c r="A43" s="4" t="n">
-        <v>5583987008152</v>
+        <v>5583981508768</v>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Rogerio</t>
+          <t>Samir</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Rogerio Cipriano Silva</t>
+          <t>Samir Said Castor Goncalves</t>
         </is>
       </c>
     </row>
     <row r="44" ht="15.75" customHeight="1" s="3">
       <c r="A44" s="4" t="n">
-        <v>5583993985481</v>
+        <v>5583993707561</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Abraao</t>
+          <t>Antonio</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Abraao Freire Leite</t>
+          <t>Antonio Pessoa Cirino</t>
         </is>
       </c>
     </row>
     <row r="45" ht="15.75" customHeight="1" s="3">
       <c r="A45" s="4" t="n">
-        <v>5583991734890</v>
+        <v>5583987008152</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Eliane</t>
+          <t>Rogerio</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Eliane Ferreira da Silva</t>
+          <t>Rogerio Cipriano Silva</t>
         </is>
       </c>
     </row>
     <row r="46" ht="15.75" customHeight="1" s="3">
       <c r="A46" s="4" t="n">
-        <v>5583986210860</v>
+        <v>5583993985481</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Alyahn</t>
+          <t>Abraao</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Alyahn Gomes de Oliveira</t>
+          <t>Abraao Freire Leite</t>
         </is>
       </c>
     </row>
     <row r="47" ht="15.75" customHeight="1" s="3">
       <c r="A47" s="4" t="n">
-        <v>5583988861453</v>
+        <v>5583991734890</v>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Luiz</t>
+          <t>Eliane</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Luiz de Araujo Santos</t>
+          <t>Eliane Ferreira da Silva</t>
         </is>
       </c>
     </row>
     <row r="48" ht="15.75" customHeight="1" s="3">
       <c r="A48" s="4" t="n">
-        <v>5583988135778</v>
+        <v>5583986210860</v>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Wanberto</t>
+          <t>Alyahn</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Wanberto da Silva Oliveira</t>
+          <t>Alyahn Gomes de Oliveira</t>
         </is>
       </c>
     </row>
     <row r="49" ht="15.75" customHeight="1" s="3">
       <c r="A49" s="4" t="n">
-        <v>5583987752644</v>
+        <v>5583988861453</v>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Lilian</t>
+          <t>Luiz</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Lilian Gavioli Guerra do Nascimento</t>
+          <t>Luiz de Araujo Santos</t>
         </is>
       </c>
     </row>
     <row r="50" ht="15.75" customHeight="1" s="3">
       <c r="A50" s="4" t="n">
-        <v>5583999412481</v>
+        <v>5583988135778</v>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Marcos</t>
+          <t>Wanberto</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Marcos Leao dos Santos Farias</t>
+          <t>Wanberto da Silva Oliveira</t>
         </is>
       </c>
     </row>
     <row r="51" ht="15.75" customHeight="1" s="3">
       <c r="A51" s="4" t="n">
-        <v>5583987954004</v>
+        <v>5583987752644</v>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Aglai</t>
+          <t>Lilian</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Aglai de Araujo Alves</t>
+          <t>Lilian Gavioli Guerra do Nascimento</t>
         </is>
       </c>
     </row>

</xml_diff>